<commit_message>
Don't need to create latitude and longitute or create any data as this sheet is already ready
</commit_message>
<xml_diff>
--- a/Data/raw/lga_addresses.xlsx
+++ b/Data/raw/lga_addresses.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\BCom &amp; BEcon\S1 26\Data and evidence in economics\ECC3479 Median Rent\ECC3479-Median-Rent\Data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1348783-4919-46B1-9773-2BBDD8161FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A5AB099-1C2C-4BB0-B738-6DD07129C416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4770" yWindow="2810" windowWidth="14400" windowHeight="7270" firstSheet="1" activeTab="1" xr2:uid="{48D51EB9-9E87-47CF-A263-C3A5A67B8DEA}"/>
+    <workbookView xWindow="3250" yWindow="1440" windowWidth="14400" windowHeight="7270" firstSheet="1" activeTab="1" xr2:uid="{48D51EB9-9E87-47CF-A263-C3A5A67B8DEA}"/>
   </bookViews>
   <sheets>
     <sheet name="Rent" sheetId="1" r:id="rId1"/>
@@ -648,9 +648,6 @@
     <t>Non-Metro</t>
   </si>
   <si>
-    <t>Suburb</t>
-  </si>
-  <si>
     <t>Level 3, 1 Flintoff Street, Greensborough, VIC 3088</t>
   </si>
   <si>
@@ -751,6 +748,9 @@
   </si>
   <si>
     <t>Address</t>
+  </si>
+  <si>
+    <t>Local Government Area</t>
   </si>
 </sst>
 </file>
@@ -61311,16 +61311,16 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="17" t="s">
-        <v>203</v>
+        <v>237</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C1" s="17" t="s">
+        <v>234</v>
+      </c>
+      <c r="D1" s="17" t="s">
         <v>235</v>
-      </c>
-      <c r="D1" s="17" t="s">
-        <v>236</v>
       </c>
       <c r="E1" s="17"/>
       <c r="F1" s="17"/>
@@ -61335,7 +61335,7 @@
         <v>166</v>
       </c>
       <c r="B2" s="23" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C2">
         <v>17.510000000000002</v>
@@ -61349,7 +61349,7 @@
         <v>167</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C3">
         <v>12.13</v>
@@ -61363,7 +61363,7 @@
         <v>168</v>
       </c>
       <c r="B4" s="23" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C4">
         <v>9.14</v>
@@ -61377,7 +61377,7 @@
         <v>169</v>
       </c>
       <c r="B5" s="23" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C5">
         <v>12.87</v>
@@ -61391,7 +61391,7 @@
         <v>145</v>
       </c>
       <c r="B6" s="23" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C6">
         <v>15.37</v>
@@ -61405,7 +61405,7 @@
         <v>170</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C7">
         <v>5.7</v>
@@ -61419,7 +61419,7 @@
         <v>171</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C8">
         <v>0.23</v>
@@ -61433,7 +61433,7 @@
         <v>172</v>
       </c>
       <c r="B9" s="23" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C9">
         <v>36.32</v>
@@ -61447,7 +61447,7 @@
         <v>173</v>
       </c>
       <c r="B10" s="25" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C10">
         <v>8.2799999999999994</v>
@@ -61461,7 +61461,7 @@
         <v>174</v>
       </c>
       <c r="B11" s="24" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C11">
         <v>6.65</v>
@@ -61475,7 +61475,7 @@
         <v>175</v>
       </c>
       <c r="B12" s="23" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C12">
         <v>18.940000000000001</v>
@@ -61489,7 +61489,7 @@
         <v>176</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C13">
         <v>36.340000000000003</v>
@@ -61503,7 +61503,7 @@
         <v>177</v>
       </c>
       <c r="B14" s="23" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C14">
         <v>27.35</v>
@@ -61517,7 +61517,7 @@
         <v>178</v>
       </c>
       <c r="B15" s="23" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C15">
         <v>3.25</v>
@@ -61531,7 +61531,7 @@
         <v>180</v>
       </c>
       <c r="B16" s="26" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C16">
         <v>8.61</v>
@@ -61545,7 +61545,7 @@
         <v>181</v>
       </c>
       <c r="B17" s="24" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C17">
         <v>25.51</v>
@@ -61559,7 +61559,7 @@
         <v>182</v>
       </c>
       <c r="B18" s="24" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C18">
         <v>15.18</v>
@@ -61573,7 +61573,7 @@
         <v>183</v>
       </c>
       <c r="B19" s="24" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C19">
         <v>24.24</v>
@@ -61587,7 +61587,7 @@
         <v>184</v>
       </c>
       <c r="B20" s="23" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="C20">
         <v>19.14</v>
@@ -61601,7 +61601,7 @@
         <v>185</v>
       </c>
       <c r="B21" s="23" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C21">
         <v>19.079999999999998</v>
@@ -61615,7 +61615,7 @@
         <v>186</v>
       </c>
       <c r="B22" s="23" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C22">
         <v>34.81</v>
@@ -61629,7 +61629,7 @@
         <v>188</v>
       </c>
       <c r="B23" s="23" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C23">
         <v>16.739999999999998</v>
@@ -61643,7 +61643,7 @@
         <v>189</v>
       </c>
       <c r="B24" s="23" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C24">
         <v>48.28</v>
@@ -61657,7 +61657,7 @@
         <v>190</v>
       </c>
       <c r="B25" s="23" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C25">
         <v>37.33</v>
@@ -61671,7 +61671,7 @@
         <v>191</v>
       </c>
       <c r="B26" s="24" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C26" s="24">
         <v>39.47</v>
@@ -61685,7 +61685,7 @@
         <v>192</v>
       </c>
       <c r="B27" s="24" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C27">
         <v>8.9</v>
@@ -61699,7 +61699,7 @@
         <v>193</v>
       </c>
       <c r="B28" s="24" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C28">
         <v>29.25</v>
@@ -61713,7 +61713,7 @@
         <v>194</v>
       </c>
       <c r="B29" s="24" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C29">
         <v>18.71</v>
@@ -61727,7 +61727,7 @@
         <v>195</v>
       </c>
       <c r="B30" s="24" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C30">
         <v>62.11</v>
@@ -61741,7 +61741,7 @@
         <v>196</v>
       </c>
       <c r="B31" s="24" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C31">
         <v>6.31</v>
@@ -61755,7 +61755,7 @@
         <v>197</v>
       </c>
       <c r="B32" s="24" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C32">
         <v>7.31</v>
@@ -61785,6 +61785,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C4E107E29A1E264B9A1CFEA965011E0D" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1ec48f4486fdb89687bf3303574062fd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="4a224ada-90ca-4535-81d1-bcf56270707c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="0423481d03504a0139e909c6bd888b31" ns3:_="">
     <xsd:import namespace="4a224ada-90ca-4535-81d1-bcf56270707c"/>
@@ -61928,12 +61934,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{73EAE720-B65E-4DFC-B754-7D2A006249B6}">
   <ds:schemaRefs>
@@ -61943,6 +61943,22 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C16EC79B-24B0-42FF-BF1A-BE13CEAA4E1B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="4a224ada-90ca-4535-81d1-bcf56270707c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{15280842-30E5-4987-8D23-E0CEEFC64C26}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -61958,20 +61974,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C16EC79B-24B0-42FF-BF1A-BE13CEAA4E1B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="4a224ada-90ca-4535-81d1-bcf56270707c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>